<commit_message>
Fix episodes 4-10 to read Excel inputs
</commit_message>
<xml_diff>
--- a/第10回_RAG/excel_rag_demo.xlsx
+++ b/第10回_RAG/excel_rag_demo.xlsx
@@ -100,7 +100,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -122,11 +122,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00D8DEE9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -155,6 +161,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -533,7 +542,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Excelで体験する言語モデルのしくみ 第10回 RAG</t>
         </is>
@@ -646,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="170" customWidth="1" min="1" max="1"/>
@@ -658,298 +667,294 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>11_PYTHON_CODE: Python in Excelへ貼り付けるコード</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>外部 .py ファイルと同じ内容です。Excelの入力表を xl(...) で参照します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" t="inlineStr">
         <is>
           <t>import pandas as pd</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="3" t="inlineStr"/>
-    </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>question = "Python in ExcelでRAG教材を外部APIなしで動かすとき、検索スコア、根拠、回答案の何を確認すればよいですか"</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>top_k = 3</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>input_source_df = xl("'01_INPUT'!A6:C9", headers=True).dropna(how="all")</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>score_threshold = 0.18</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>documents_source_df = xl("'02_DOCUMENTS'!A5:D12", headers=True).dropna(how="all")</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>query_features = [('python', 1.0), ('excel', 1.0), ('rag', 1.4), ('外部api', 1.2), ('検索', 1.1), ('根拠', 1.2), ('回答', 0.9), ('教材', 0.8)]</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>query_features_source_df = xl("'03_QUERY_FEATURES'!A5:C13", headers=True).dropna(how="all")</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>documents = [</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D01","title":"RAGの基本","text":"RAGは質問に近い外部資料を検索し、その根拠を回答に添える構成です。","tags":"rag,検索,根拠,回答"},</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>settings = dict(zip(input_source_df["parameter"].astype(str), input_source_df["value"]))</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D02","title":"Python in Excel","text":"Python in Excelではコード実行はMicrosoft Cloud上で行われ、実行には対応するMicrosoft 365環境とインターネット接続が必要です。","tags":"python,excel,実行環境,cloud"},</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>question = str(settings.get("question", ""))</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D03","title":"教材用の簡略化","text":"この教材では外部APIを呼ばず、キーワード重みによる簡易スコアで検索の流れを確認します。","tags":"教材,外部api,検索,簡略化"},</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>top_k = int(float(settings.get("top_k", 3)))</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D04","title":"生成の扱い","text":"回答生成はLLM APIではなく、上位文書の根拠文を使ったテンプレートで組み立てます。","tags":"回答,根拠,テンプレート,llm"},</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>score_threshold = float(settings.get("score_threshold", 0.18))</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D05","title":"前回との違い","text":"Backpropagationは内部重みを更新しますが、RAGは学習済みモデルの外側に資料をつなぎます。","tags":"backpropagation,rag,外部資料,重み"},</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>query_features = [</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D06","title":"本格RAGで必要なもの","text":"実サービスではembedding、ベクトルDB、chunking、reranker、プロンプト設計、権限管理が重要です。","tags":"embedding,vector,chunking,reranker"},</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (str(row["query_feature"]), float(row["weight"]))</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    {"document_id":"D07","title":"確認する表","text":"検索スコア、上位文書、根拠文、回答案を分けて見ると、どの資料を使ったか説明しやすくなります。","tags":"検索,スコア,上位文書,根拠,回答"},</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    for _, row in query_features_source_df.iterrows()</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>]</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>documents = documents_source_df[["document_id", "title", "text", "tags"]].to_dict("records")</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" t="inlineStr">
         <is>
           <t>q_terms = [term for term, weight in query_features if term.lower() in question.lower()]</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" t="inlineStr">
         <is>
           <t>max_possible = sum(weight for term, weight in query_features if term in q_terms) or 1.0</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" t="inlineStr">
         <is>
           <t>query_features_df = pd.DataFrame([{"query_feature":term,"weight":weight,"status":"queryに含まれる" if term in q_terms else "検索語として待機"} for term, weight in query_features])</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" t="inlineStr">
         <is>
           <t>documents_df = pd.DataFrame(documents)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" t="inlineStr">
         <is>
           <t>records = []</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" t="inlineStr">
         <is>
           <t>for doc in documents:</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" t="inlineStr">
         <is>
           <t xml:space="preserve">    haystack = f"{doc['title']} {doc['text']} {doc['tags']}".lower()</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">    matched = [(term, weight) for term, weight in query_features if term in q_terms and term.lower() in haystack]</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" t="inlineStr">
         <is>
           <t xml:space="preserve">    raw_score = sum(weight for term, weight in matched)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" t="inlineStr">
         <is>
           <t xml:space="preserve">    records.append({"document_id":doc["document_id"],"title":doc["title"],"matched_terms":", ".join(term for term, weight in matched) or "-","raw_score":round(raw_score,4),"score":round(raw_score/max_possible,4),"text":doc["text"]})</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" t="inlineStr">
         <is>
           <t>records = sorted(records, key=lambda row: (-row["score"], row["document_id"]))</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" t="inlineStr">
         <is>
           <t>for i, row in enumerate(records, 1):</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" t="inlineStr">
         <is>
           <t xml:space="preserve">    row["rank"] = i</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" t="inlineStr">
         <is>
           <t xml:space="preserve">    row["decision"] = "use" if i &lt;= top_k and row["score"] &gt;= score_threshold else "skip"</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" t="inlineStr">
         <is>
           <t>retrieval_score_df = pd.DataFrame(records)[["document_id","title","matched_terms","raw_score","score","rank","decision"]]</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" t="inlineStr">
         <is>
           <t>top_context_df = pd.DataFrame([{"rank":r["rank"],"document_id":r["document_id"],"title":r["title"],"score":r["score"],"evidence_text":r["text"]} for r in records if r["decision"] == "use"])</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" t="inlineStr">
         <is>
           <t>evidence = " / ".join([f"{row.document_id}: {row.evidence_text}" for row in top_context_df.itertuples()])</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" t="inlineStr">
         <is>
           <t>answer_draft_df = pd.DataFrame([{"field":"question","value":question},{"field":"evidence","value":evidence},{"field":"answer_draft","value":"外部APIを使わない教材では、質問に近い資料をキーワード重みで検索し、検索スコア、上位文書、根拠文、回答案が対応しているかを確認します。Python in Excelで実行する場合は、コード自体はAPIを呼ばなくても実行環境にはインターネット接続とMicrosoft 365環境が必要です。"},{"field":"caution","value":"これは教材用の簡易RAGです。embedding、ベクトルDB、reranker、LLM APIによる生成は扱いません。"}])</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" t="inlineStr">
         <is>
           <t>rag_flow_df = pd.DataFrame([{"step":1,"stage":"query","meaning":"質問文から検索語を見る"},{"step":2,"stage":"retrieve","meaning":"文書ごとに一致語と重みを足す"},{"step":3,"stage":"context","meaning":"top_kとthresholdで根拠文を選ぶ"},{"step":4,"stage":"answer","meaning":"根拠文から回答案を組み立てる"}])</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" t="inlineStr">
         <is>
           <t>result_df = retrieval_score_df</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" t="inlineStr">
         <is>
           <t># result_df = documents_df</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" t="inlineStr">
         <is>
           <t># result_df = query_features_df</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" t="inlineStr">
         <is>
           <t># result_df = top_context_df</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="24" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" t="inlineStr">
         <is>
           <t># result_df = answer_draft_df</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="24" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" t="inlineStr">
         <is>
           <t># result_df = rag_flow_df</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>result_df</t>
         </is>
@@ -981,7 +986,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>12_TROUBLE: よくある確認点</t>
         </is>
@@ -1006,7 +1011,7 @@
           <t>よくある確認点</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1095,7 +1100,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>13_SERIES_ROADMAP</t>
         </is>
@@ -1122,8 +1127,8 @@
           <t>全10回ロードマップ</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1343,7 +1348,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>01_INPUT: RAG検索の入力</t>
         </is>
@@ -1376,15 +1381,15 @@
           <t>質問、検索件数、しきい値を入口にして、どの資料が根拠に選ばれるかを確認します。</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="n"/>
@@ -1404,8 +1409,8 @@
           <t>RAG demo input</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
@@ -1534,7 +1539,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>02_DOCUMENTS: 外部資料として参照する文書</t>
         </is>
@@ -1563,9 +1568,9 @@
           <t>検索対象の小さな資料表</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1770,7 +1775,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>03_QUERY_FEATURES: 質問から見る検索語と重み</t>
         </is>
@@ -1797,8 +1802,8 @@
           <t>query features</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1965,7 +1970,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>04_RETRIEVAL_SCORE: 文書ごとの検索スコア</t>
         </is>
@@ -2001,12 +2006,12 @@
           <t>retrieval score</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2289,7 +2294,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>05_TOP_CONTEXT: 回答に使う根拠文</t>
         </is>
@@ -2320,10 +2325,10 @@
           <t>top context</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2448,7 +2453,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>06_ANSWER_DRAFT: 根拠から作る回答案</t>
         </is>
@@ -2473,7 +2478,7 @@
           <t>answer draft</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2562,7 +2567,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>07_RAG_FLOW: queryからanswerまで</t>
         </is>
@@ -2589,8 +2594,8 @@
           <t>RAG flow</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2704,7 +2709,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>10_RUN_PYTHON: Python in Excel 実行手順</t>
         </is>
@@ -2729,7 +2734,7 @@
           <t>実行手順</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Clean public Office metadata
</commit_message>
<xml_diff>
--- a/第10回_RAG/excel_rag_demo.xlsx
+++ b/第10回_RAG/excel_rag_demo.xlsx
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -164,6 +164,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -655,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="170" customWidth="1" min="1" max="1"/>
@@ -688,9 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5" ht="24" customHeight="1"/>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
@@ -712,9 +716,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9" ht="24" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
@@ -1006,7 +1008,7 @@
       <c r="B3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>よくある確認点</t>
         </is>
@@ -1122,7 +1124,7 @@
       <c r="C3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>全10回ロードマップ</t>
         </is>
@@ -1376,7 +1378,7 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>質問、検索件数、しきい値を入口にして、どの資料が根拠に選ばれるかを確認します。</t>
         </is>
@@ -1404,7 +1406,7 @@
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>RAG demo input</t>
         </is>
@@ -1563,7 +1565,7 @@
       <c r="D3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>検索対象の小さな資料表</t>
         </is>
@@ -1797,7 +1799,7 @@
       <c r="C3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>query features</t>
         </is>
@@ -2001,7 +2003,7 @@
       <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>retrieval score</t>
         </is>
@@ -2320,7 +2322,7 @@
       <c r="E3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>top context</t>
         </is>
@@ -2473,7 +2475,7 @@
       <c r="B3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>answer draft</t>
         </is>
@@ -2589,7 +2591,7 @@
       <c r="C3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>RAG flow</t>
         </is>
@@ -2729,7 +2731,7 @@
       <c r="B3" s="3" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>実行手順</t>
         </is>

</xml_diff>